<commit_message>
Repository cleanup and deployment preparation
</commit_message>
<xml_diff>
--- a/Amazon Financial Intelligence/data/Amazon_raw_data.xlsx
+++ b/Amazon Financial Intelligence/data/Amazon_raw_data.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\shivaum\OneDrive\Desktop\Data Science\Business Analytics Project\Amazon Financial Intelligence\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\shivaum\OneDrive\Desktop\Coding\Projects\Business Analytics Project\Amazon Financial Intelligence\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0FF2F76A-F027-4833-B951-99225A612D37}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{643C31BA-01C9-4F0F-ABCE-0C5C36B5A5CA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-90" yWindow="0" windowWidth="12980" windowHeight="15370" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="12710" yWindow="0" windowWidth="12980" windowHeight="15370" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Year,Total_Revenue,Operating_In" sheetId="2" r:id="rId1"/>

</xml_diff>